<commit_message>
Build workbook-driven Sanity listicle template
</commit_message>
<xml_diff>
--- a/outputs/01a0a89b-ff01-7c02-b12a-008d8164e9b1/MaximusLabs listicle feed updated.xlsx
+++ b/outputs/01a0a89b-ff01-7c02-b12a-008d8164e9b1/MaximusLabs listicle feed updated.xlsx
@@ -2,27 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc4d131a694524547"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="players" sheetId="2" r:id="R7cb4ef6149d54326"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="directions" sheetId="3" r:id="R7f088f2c98f745b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="service_axis" sheetId="4" r:id="R67fe4290a0be4281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coverage" sheetId="5" r:id="R14ac6a18028b4e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vertical_services" sheetId="6" r:id="R4738956cdc8946f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vertical_meta" sheetId="7" r:id="R2583a704b57a4261"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="quick_answer" sheetId="8" r:id="R08d359d3c188429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratings" sheetId="9" r:id="R1a835f2276d94ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reviews" sheetId="10" r:id="R66dac8869b7c4efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cases" sheetId="11" r:id="R0d6e28da4ee74e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="portfolio" sheetId="12" r:id="R869f70402c4f4f7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="listings" sheetId="13" r:id="R93bf1c574cc24a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="below_the_line" sheetId="14" r:id="R138a01e1f3be4e26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="15" r:id="R8d48a28025444231"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="page_spec" sheetId="16" r:id="R0219f83e556540a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="listicle_pages" sheetId="17" r:id="R474b59c0c0d6483b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="assessment_keys" sheetId="18" r:id="Rb8e40efa3d7645b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="methodology" sheetId="19" r:id="R9ae51a028b7d4dc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="20" r:id="Rbb07b95e925b485a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="review_notes" sheetId="21" r:id="R32aa30fd3d544d0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd6a6f83358a94ad7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="players" sheetId="2" r:id="Rb4d108b11f41403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="directions" sheetId="3" r:id="Rfff6e578d0064991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="service_axis" sheetId="4" r:id="Rdefa5bd6228949b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coverage" sheetId="5" r:id="Red5612652e9e44df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vertical_services" sheetId="6" r:id="Ra8820d12219f4211"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vertical_meta" sheetId="7" r:id="R3778341df5f3479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="quick_answer" sheetId="8" r:id="Rf8698c2caee2476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratings" sheetId="9" r:id="Ra8fead26f2284864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reviews" sheetId="10" r:id="Rbf46da96f7174685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cases" sheetId="11" r:id="R39633a1c26534bf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="portfolio" sheetId="12" r:id="Rc77ecbaccd34471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="listings" sheetId="13" r:id="R49fc2f4633b34281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="below_the_line" sheetId="14" r:id="R1840a177f8534554"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="15" r:id="R35ecafa5def34b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="page_spec" sheetId="16" r:id="R10c8b75c687b42e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="listicle_pages" sheetId="17" r:id="Rd39b90274a7549c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="assessment_keys" sheetId="18" r:id="R25686d8517c34b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="methodology" sheetId="19" r:id="Rb6398b4596194ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="20" r:id="Ra6e996ebdda64e73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="review_notes" sheetId="21" r:id="R07d6eaf246c84432"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="writing_memory" sheetId="22" r:id="R99def1f571e843b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,7 +37,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -76,8 +77,25 @@
       <x:color rgb="FF111111"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF111827"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF4B5563"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -92,8 +110,13 @@
         <x:fgColor rgb="FF000000"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -123,11 +146,67 @@
         <x:color rgb="FFD9D9D9"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF9CA3AF"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF111111"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF111111"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF111111"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF111111"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF111111"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF111111"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF111111"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF111111"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFE5E7EB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFE5E7EB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE5E7EB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFE5E7EB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyAlignment="1">
@@ -186,6 +265,66 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -722,8 +861,12 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23"/>
-      <x:c r="B23"/>
+      <x:c r="A23" s="25" t="str">
+        <x:v>writing_memory</x:v>
+      </x:c>
+      <x:c r="B23" s="26" t="str">
+        <x:v>Reusable writing rules and the fixed page-to-Sanity mapping for every listicle.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="5" t="str">
@@ -10792,6 +10935,503 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="72" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="27" t="str">
+        <x:v>Listicle writing memory</x:v>
+      </x:c>
+      <x:c r="B1" s="27"/>
+      <x:c r="C1" s="27"/>
+      <x:c r="D1" s="27"/>
+      <x:c r="E1" s="27"/>
+      <x:c r="F1" s="27"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="29" t="str">
+        <x:v>Rules and field mappings used to turn one workbook row set into the fixed MaximusLabs listicle template.</x:v>
+      </x:c>
+      <x:c r="B2" s="29"/>
+      <x:c r="C2" s="29"/>
+      <x:c r="D2" s="29"/>
+      <x:c r="E2" s="29"/>
+      <x:c r="F2" s="29"/>
+    </x:row>
+    <x:row r="4" ht="28" hidden="0" customHeight="1">
+      <x:c r="A4" s="41" t="str">
+        <x:v>scope</x:v>
+      </x:c>
+      <x:c r="B4" s="42" t="str">
+        <x:v>rule_order</x:v>
+      </x:c>
+      <x:c r="C4" s="42" t="str">
+        <x:v>instruction</x:v>
+      </x:c>
+      <x:c r="D4" s="42" t="str">
+        <x:v>sanity_target</x:v>
+      </x:c>
+      <x:c r="E4" s="42" t="str">
+        <x:v>source_tab</x:v>
+      </x:c>
+      <x:c r="F4" s="43" t="str">
+        <x:v>required</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>global</x:v>
+      </x:c>
+      <x:c r="B5" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>The workbook is the source of truth. Render from approved workbook data, never from an earlier draft.</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>all imported documents</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>README</x:v>
+      </x:c>
+      <x:c r="F5" s="48" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="46" t="str">
+        <x:v>global</x:v>
+      </x:c>
+      <x:c r="B6" s="49" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C6" s="46" t="str">
+        <x:v>Use player_id as the reusable agency join key across listings.</x:v>
+      </x:c>
+      <x:c r="D6" s="46" t="str">
+        <x:v>agency.playerId and references</x:v>
+      </x:c>
+      <x:c r="E6" s="46" t="str">
+        <x:v>README</x:v>
+      </x:c>
+      <x:c r="F6" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="46" t="str">
+        <x:v>global</x:v>
+      </x:c>
+      <x:c r="B7" s="49" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C7" s="46" t="str">
+        <x:v>Treat pipe-separated cell values as ordered arrays.</x:v>
+      </x:c>
+      <x:c r="D7" s="46" t="str">
+        <x:v>array fields</x:v>
+      </x:c>
+      <x:c r="E7" s="46" t="str">
+        <x:v>README</x:v>
+      </x:c>
+      <x:c r="F7" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="46" t="str">
+        <x:v>global</x:v>
+      </x:c>
+      <x:c r="B8" s="49" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C8" s="46" t="str">
+        <x:v>Use 'Not published' for unknown evidence. Do not invent missing claims.</x:v>
+      </x:c>
+      <x:c r="D8" s="46" t="str">
+        <x:v>evidence fields</x:v>
+      </x:c>
+      <x:c r="E8" s="46" t="str">
+        <x:v>README</x:v>
+      </x:c>
+      <x:c r="F8" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="46" t="str">
+        <x:v>global</x:v>
+      </x:c>
+      <x:c r="B9" s="49" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C9" s="46" t="str">
+        <x:v>Reuse an existing player and vertical. Enrich only the missing vertical records.</x:v>
+      </x:c>
+      <x:c r="D9" s="46" t="str">
+        <x:v>agency.verticalProfiles</x:v>
+      </x:c>
+      <x:c r="E9" s="46" t="str">
+        <x:v>README</x:v>
+      </x:c>
+      <x:c r="F9" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="46" t="str">
+        <x:v>global</x:v>
+      </x:c>
+      <x:c r="B10" s="49" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C10" s="46" t="str">
+        <x:v>Create a new service axis for every new vertical. Do not reuse another vertical taxonomy.</x:v>
+      </x:c>
+      <x:c r="D10" s="46" t="str">
+        <x:v>listiclePage.serviceAxis</x:v>
+      </x:c>
+      <x:c r="E10" s="46" t="str">
+        <x:v>README</x:v>
+      </x:c>
+      <x:c r="F10" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
+      <x:c r="A11" s="46" t="str">
+        <x:v>global</x:v>
+      </x:c>
+      <x:c r="B11" s="49" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C11" s="46" t="str">
+        <x:v>Keep capability and industry scores in Sanity for auditability, but do not render them as editorial claims.</x:v>
+      </x:c>
+      <x:c r="D11" s="46" t="str">
+        <x:v>listicleEntry scores</x:v>
+      </x:c>
+      <x:c r="E11" s="46" t="str">
+        <x:v>listings</x:v>
+      </x:c>
+      <x:c r="F11" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
+      <x:c r="A12" s="46" t="str">
+        <x:v>Top nav</x:v>
+      </x:c>
+      <x:c r="B12" s="49" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="46" t="str">
+        <x:v>Keep the fixed navigation: Directory, Methodology, Compare all, Studio, and desktop/mobile preview.</x:v>
+      </x:c>
+      <x:c r="D12" s="46" t="str">
+        <x:v>React template only</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="str">
+        <x:v>page_spec</x:v>
+      </x:c>
+      <x:c r="F12" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="46" t="str">
+        <x:v>Breadcrumb row</x:v>
+      </x:c>
+      <x:c r="B13" s="49" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C13" s="46" t="str">
+        <x:v>Show publisher, directory, vertical, review date, and evaluated-firm count.</x:v>
+      </x:c>
+      <x:c r="D13" s="46" t="str">
+        <x:v>publisherName, verticalLabel, reviewedAt, entries</x:v>
+      </x:c>
+      <x:c r="E13" s="46" t="str">
+        <x:v>page_spec</x:v>
+      </x:c>
+      <x:c r="F13" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" hidden="0" customHeight="1">
+      <x:c r="A14" s="46" t="str">
+        <x:v>Headline</x:v>
+      </x:c>
+      <x:c r="B14" s="49" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C14" s="46" t="str">
+        <x:v>Use the approved workbook headline and year. Do not generate a replacement title during import.</x:v>
+      </x:c>
+      <x:c r="D14" s="46" t="str">
+        <x:v>title, year</x:v>
+      </x:c>
+      <x:c r="E14" s="46" t="str">
+        <x:v>listicle_pages</x:v>
+      </x:c>
+      <x:c r="F14" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="46" t="str">
+        <x:v>Dek</x:v>
+      </x:c>
+      <x:c r="B15" s="49" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C15" s="46" t="str">
+        <x:v>Use one sentence explaining what the list evaluates and the evidence basis.</x:v>
+      </x:c>
+      <x:c r="D15" s="46" t="str">
+        <x:v>dek</x:v>
+      </x:c>
+      <x:c r="E15" s="46" t="str">
+        <x:v>listicle_pages</x:v>
+      </x:c>
+      <x:c r="F15" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="46" t="str">
+        <x:v>Publisher disclosure</x:v>
+      </x:c>
+      <x:c r="B16" s="49" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C16" s="46" t="str">
+        <x:v>State that MaximusLabs competes with listed firms and direct readers to the methodology.</x:v>
+      </x:c>
+      <x:c r="D16" s="46" t="str">
+        <x:v>publisherDisclosure</x:v>
+      </x:c>
+      <x:c r="E16" s="46" t="str">
+        <x:v>listicle_pages</x:v>
+      </x:c>
+      <x:c r="F16" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="46" t="str">
+        <x:v>Three-up key</x:v>
+      </x:c>
+      <x:c r="B17" s="49" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C17" s="46" t="str">
+        <x:v>Use exactly three assessment blocks in workbook order.</x:v>
+      </x:c>
+      <x:c r="D17" s="46" t="str">
+        <x:v>assessmentKeys</x:v>
+      </x:c>
+      <x:c r="E17" s="46" t="str">
+        <x:v>assessment_keys</x:v>
+      </x:c>
+      <x:c r="F17" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="46" t="str">
+        <x:v>Quick answer panel</x:v>
+      </x:c>
+      <x:c r="B18" s="49" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C18" s="46" t="str">
+        <x:v>Show the approved top five reasons and link each entry to its full card.</x:v>
+      </x:c>
+      <x:c r="D18" s="46" t="str">
+        <x:v>quickAnswers</x:v>
+      </x:c>
+      <x:c r="E18" s="46" t="str">
+        <x:v>quick_answer</x:v>
+      </x:c>
+      <x:c r="F18" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="46" t="str">
+        <x:v>Sidebar contents</x:v>
+      </x:c>
+      <x:c r="B19" s="49" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C19" s="46" t="str">
+        <x:v>Generate navigation from the ranked entries and approved comparison questions.</x:v>
+      </x:c>
+      <x:c r="D19" s="46" t="str">
+        <x:v>entries, questions</x:v>
+      </x:c>
+      <x:c r="E19" s="46" t="str">
+        <x:v>page_spec</x:v>
+      </x:c>
+      <x:c r="F19" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="46" t="str">
+        <x:v>Comparison table</x:v>
+      </x:c>
+      <x:c r="B20" s="49" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C20" s="46" t="str">
+        <x:v>Use workbook levers, clients, proof, limits, and monthly pricing.</x:v>
+      </x:c>
+      <x:c r="D20" s="46" t="str">
+        <x:v>entries and agency references</x:v>
+      </x:c>
+      <x:c r="E20" s="46" t="str">
+        <x:v>directions, players, vertical_meta</x:v>
+      </x:c>
+      <x:c r="F20" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="46" t="str">
+        <x:v>Ranked cards</x:v>
+      </x:c>
+      <x:c r="B21" s="49" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C21" s="46" t="str">
+        <x:v>Render every ranked agency with facts, ratings, services, reviews, cases, and best-for copy.</x:v>
+      </x:c>
+      <x:c r="D21" s="46" t="str">
+        <x:v>entries and agency documents</x:v>
+      </x:c>
+      <x:c r="E21" s="46" t="str">
+        <x:v>listings and agency tabs</x:v>
+      </x:c>
+      <x:c r="F21" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
+      <x:c r="A22" s="46" t="str">
+        <x:v>Methodology</x:v>
+      </x:c>
+      <x:c r="B22" s="49" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C22" s="46" t="str">
+        <x:v>Use the page-specific introduction, ordered steps, community finding, and correction.</x:v>
+      </x:c>
+      <x:c r="D22" s="46" t="str">
+        <x:v>methodologyIntro, methodologySteps, methodologyCommunityFinding, methodologyCorrection</x:v>
+      </x:c>
+      <x:c r="E22" s="46" t="str">
+        <x:v>listicle_pages, methodology</x:v>
+      </x:c>
+      <x:c r="F22" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="46" t="str">
+        <x:v>Service matrix</x:v>
+      </x:c>
+      <x:c r="B23" s="49" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C23" s="46" t="str">
+        <x:v>Use the vertical service axis and per-agency coverage marks.</x:v>
+      </x:c>
+      <x:c r="D23" s="46" t="str">
+        <x:v>serviceAxis, entries.coverage</x:v>
+      </x:c>
+      <x:c r="E23" s="46" t="str">
+        <x:v>service_axis, coverage</x:v>
+      </x:c>
+      <x:c r="F23" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="46" t="str">
+        <x:v>Comparison questions</x:v>
+      </x:c>
+      <x:c r="B24" s="49" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C24" s="46" t="str">
+        <x:v>Render the approved ordered questions and their table types.</x:v>
+      </x:c>
+      <x:c r="D24" s="46" t="str">
+        <x:v>questions</x:v>
+      </x:c>
+      <x:c r="E24" s="46" t="str">
+        <x:v>questions</x:v>
+      </x:c>
+      <x:c r="F24" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="46" t="str">
+        <x:v>Also considered</x:v>
+      </x:c>
+      <x:c r="B25" s="49" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C25" s="46" t="str">
+        <x:v>Keep researched exclusions with their reason and reconsideration condition.</x:v>
+      </x:c>
+      <x:c r="D25" s="46" t="str">
+        <x:v>alsoConsidered</x:v>
+      </x:c>
+      <x:c r="E25" s="46" t="str">
+        <x:v>below_the_line</x:v>
+      </x:c>
+      <x:c r="F25" s="49" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="24" hidden="0" customHeight="1">
+      <x:c r="A26" s="47" t="str">
+        <x:v>Footer</x:v>
+      </x:c>
+      <x:c r="B26" s="50" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C26" s="47" t="str">
+        <x:v>Repeat the disclosure, review-data note, link note, and review date.</x:v>
+      </x:c>
+      <x:c r="D26" s="47" t="str">
+        <x:v>publisherDisclosure, footerReviewNote, footerLinkNote, reviewedAt</x:v>
+      </x:c>
+      <x:c r="E26" s="47" t="str">
+        <x:v>listicle_pages</x:v>
+      </x:c>
+      <x:c r="F26" s="50" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>

</xml_diff>